<commit_message>
regionalize the deit module with scenario analysis
</commit_message>
<xml_diff>
--- a/Regionalized FeliX/Model Files/New_DietData.xlsx
+++ b/Regionalized FeliX/Model Files/New_DietData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iiasahub-my.sharepoint.com/personal/yequanliang_iiasa_ac_at/Documents/research_iiasa/Felix-Model/Regionalized FeliX/Model Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="11_5523B6F1FF37483A581E8314AEA41110AD641C97" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7681FE08-5362-48AD-90B9-6CF94B38D1B3}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="11_5523B6F1FF37483A581E8314AEA41110AD641C97" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{733BBD72-A8CC-4245-9880-EFAF47569BAE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="731" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2671,7 +2671,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
@@ -2989,6 +2989,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="203">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8579,7 +8581,7 @@
       <c r="L4" s="106">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="M4" s="48">
+      <c r="M4" s="145">
         <v>1.8</v>
       </c>
       <c r="V4" s="48">
@@ -8644,7 +8646,7 @@
       <c r="L5" s="106">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="M5" s="48">
+      <c r="M5" s="145">
         <v>5.7</v>
       </c>
       <c r="V5" s="48">
@@ -8709,7 +8711,7 @@
       <c r="L6" s="106">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="M6" s="48">
+      <c r="M6" s="145">
         <v>6.8</v>
       </c>
       <c r="V6" s="48">
@@ -8774,7 +8776,7 @@
       <c r="L7" s="106">
         <v>2E-3</v>
       </c>
-      <c r="M7" s="48">
+      <c r="M7" s="145">
         <v>1.2</v>
       </c>
       <c r="V7" s="48">
@@ -8839,7 +8841,7 @@
       <c r="L8" s="106">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M8" s="48">
+      <c r="M8" s="145">
         <v>2.2999999999999998</v>
       </c>
       <c r="N8">
@@ -8920,7 +8922,7 @@
       <c r="L9" s="106">
         <v>2.3E-3</v>
       </c>
-      <c r="M9" s="48">
+      <c r="M9" s="145">
         <v>48</v>
       </c>
       <c r="N9">
@@ -9001,7 +9003,7 @@
       <c r="L10" s="106">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="M10" s="48">
+      <c r="M10" s="145">
         <v>8.1999999999999993</v>
       </c>
       <c r="N10">
@@ -9082,7 +9084,7 @@
       <c r="L11" s="106">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="M11" s="48">
+      <c r="M11" s="145">
         <v>26</v>
       </c>
       <c r="N11">
@@ -9140,8 +9142,10 @@
       <c r="H12" s="92">
         <v>1.52604801675541</v>
       </c>
+      <c r="M12" s="48"/>
     </row>
     <row r="13" spans="1:28">
+      <c r="F13" s="145"/>
       <c r="H13">
         <f>250*0.6/D12</f>
         <v>6.8306010928961755E-2</v>
@@ -9365,6 +9369,7 @@
       <c r="A20" s="89" t="s">
         <v>90</v>
       </c>
+      <c r="B20" s="146"/>
       <c r="X20" s="89" t="s">
         <v>185</v>
       </c>

</xml_diff>